<commit_message>
Corrected the thickness of Acrylic Sheets in BOM
</commit_message>
<xml_diff>
--- a/BOM/BillOfMaterials_v2.xlsx
+++ b/BOM/BillOfMaterials_v2.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11214"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A2AC89B-D598-6D40-A157-ABABCDC4630C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFD86198-E1C8-3B4F-8192-DBC1B78A10D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3560" yWindow="2860" windowWidth="34400" windowHeight="23400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3560" yWindow="2860" windowWidth="34400" windowHeight="23400" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
@@ -641,7 +641,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -669,10 +669,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -979,7 +975,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.5" bestFit="1" customWidth="1"/>
@@ -1269,7 +1265,7 @@
         <v>118</v>
       </c>
       <c r="F13" s="2">
-        <f>C13*D13</f>
+        <f t="shared" ref="F13:F18" si="2">C13*D13</f>
         <v>38.97</v>
       </c>
       <c r="G13" s="2" t="s">
@@ -1281,7 +1277,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
-        <f>A13+1</f>
+        <f t="shared" ref="A14:A19" si="3">A13+1</f>
         <v>2</v>
       </c>
       <c r="B14" s="2" t="s">
@@ -1297,7 +1293,7 @@
         <v>124</v>
       </c>
       <c r="F14" s="2">
-        <f>C14*D14</f>
+        <f t="shared" si="2"/>
         <v>19.88</v>
       </c>
       <c r="G14" s="2" t="s">
@@ -1309,7 +1305,7 @@
     </row>
     <row r="15" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <f>A14+1</f>
+        <f t="shared" si="3"/>
         <v>3</v>
       </c>
       <c r="B15" s="4" t="s">
@@ -1325,7 +1321,7 @@
         <v>126</v>
       </c>
       <c r="F15" s="2">
-        <f>C15*D15</f>
+        <f t="shared" si="2"/>
         <v>6.89</v>
       </c>
       <c r="G15" s="2" t="s">
@@ -1337,7 +1333,7 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <f>A15+1</f>
+        <f t="shared" si="3"/>
         <v>4</v>
       </c>
       <c r="B16" s="2" t="s">
@@ -1353,7 +1349,7 @@
         <v>128</v>
       </c>
       <c r="F16" s="2">
-        <f>C16*D16</f>
+        <f t="shared" si="2"/>
         <v>6.99</v>
       </c>
       <c r="G16" s="2" t="s">
@@ -1365,7 +1361,7 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <f>A16+1</f>
+        <f t="shared" si="3"/>
         <v>5</v>
       </c>
       <c r="B17" s="2" t="s">
@@ -1381,7 +1377,7 @@
         <v>134</v>
       </c>
       <c r="F17" s="2">
-        <f>C17*D17</f>
+        <f t="shared" si="2"/>
         <v>8.99</v>
       </c>
       <c r="G17" s="2" t="s">
@@ -1393,7 +1389,7 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <f>A17+1</f>
+        <f t="shared" si="3"/>
         <v>6</v>
       </c>
       <c r="B18" s="2" t="s">
@@ -1409,7 +1405,7 @@
         <v>130</v>
       </c>
       <c r="F18" s="2">
-        <f>C18*D18</f>
+        <f t="shared" si="2"/>
         <v>7.49</v>
       </c>
       <c r="G18" s="2" t="s">
@@ -1421,7 +1417,7 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <f>A18+1</f>
+        <f t="shared" si="3"/>
         <v>7</v>
       </c>
       <c r="B19" s="2" t="s">
@@ -1447,13 +1443,7 @@
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A20" s="20"/>
-      <c r="B20" s="21"/>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
-      <c r="E20" s="20"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="20"/>
+      <c r="B20" s="5"/>
       <c r="H20" s="6"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
@@ -1539,7 +1529,7 @@
         <v>67</v>
       </c>
       <c r="F25" s="2">
-        <f t="shared" ref="F25:F26" si="2">C25*D25</f>
+        <f t="shared" ref="F25:F26" si="4">C25*D25</f>
         <v>17.95</v>
       </c>
       <c r="G25" s="2" t="s">
@@ -1567,7 +1557,7 @@
         <v>71</v>
       </c>
       <c r="F26" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>3.95</v>
       </c>
       <c r="G26" s="2" t="s">
@@ -1739,7 +1729,7 @@
         <v>50</v>
       </c>
       <c r="F36" s="2">
-        <f t="shared" ref="F36:F44" si="3">C36*D36</f>
+        <f t="shared" ref="F36:F44" si="5">C36*D36</f>
         <v>5.14</v>
       </c>
       <c r="G36" s="2" t="s">
@@ -1762,7 +1752,7 @@
       </c>
       <c r="E37" s="2"/>
       <c r="F37" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>9.65</v>
       </c>
       <c r="G37" s="2" t="s">
@@ -1787,7 +1777,7 @@
         <v>96</v>
       </c>
       <c r="F38" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>9.65</v>
       </c>
       <c r="G38" s="2" t="s">
@@ -1812,7 +1802,7 @@
         <v>84</v>
       </c>
       <c r="F39" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>9.99</v>
       </c>
       <c r="G39" s="2" t="s">
@@ -1837,7 +1827,7 @@
         <v>88</v>
       </c>
       <c r="F40" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>15.99</v>
       </c>
       <c r="G40" s="2" t="s">
@@ -1862,7 +1852,7 @@
         <v>91</v>
       </c>
       <c r="F41" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>29.98</v>
       </c>
       <c r="G41" s="2" t="s">
@@ -1887,7 +1877,7 @@
         <v>104</v>
       </c>
       <c r="F42" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>6.2</v>
       </c>
       <c r="G42" s="2" t="s">
@@ -1912,7 +1902,7 @@
         <v>103</v>
       </c>
       <c r="F43" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>6.41</v>
       </c>
       <c r="G43" s="2" t="s">
@@ -1937,7 +1927,7 @@
         <v>107</v>
       </c>
       <c r="F44" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>3.69</v>
       </c>
       <c r="G44" s="2" t="s">
@@ -2175,175 +2165,26 @@
         <v>644.02999999999986</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A60" s="20"/>
-      <c r="B60" s="20"/>
-      <c r="C60" s="20"/>
-      <c r="D60" s="20"/>
-      <c r="E60" s="20"/>
-      <c r="F60" s="20"/>
-      <c r="G60" s="20"/>
-      <c r="H60" s="20"/>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A61" s="20"/>
-      <c r="B61" s="20"/>
-      <c r="C61" s="20"/>
-      <c r="D61" s="20"/>
-      <c r="E61" s="20"/>
-      <c r="F61" s="20"/>
-      <c r="G61" s="20"/>
-      <c r="H61" s="20"/>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A62" s="20"/>
-      <c r="B62" s="20"/>
-      <c r="C62" s="20"/>
-      <c r="D62" s="20"/>
-      <c r="E62" s="20"/>
-      <c r="F62" s="20"/>
-      <c r="G62" s="20"/>
-      <c r="H62" s="20"/>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A63" s="20"/>
-      <c r="B63" s="20"/>
-      <c r="C63" s="20"/>
-      <c r="D63" s="20"/>
-      <c r="E63" s="20"/>
-      <c r="F63" s="20"/>
-      <c r="G63" s="20"/>
-      <c r="H63" s="20"/>
-    </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A64" s="20"/>
-      <c r="B64" s="20"/>
-      <c r="C64" s="20"/>
-      <c r="D64" s="20"/>
-      <c r="E64" s="20"/>
-      <c r="F64" s="20"/>
-      <c r="G64" s="20"/>
-      <c r="H64" s="20"/>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A65" s="20"/>
-      <c r="B65" s="20"/>
-      <c r="C65" s="20"/>
-      <c r="D65" s="20"/>
-      <c r="E65" s="20"/>
-      <c r="F65" s="20"/>
-      <c r="G65" s="20"/>
-      <c r="H65" s="20"/>
-    </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A66" s="20"/>
-      <c r="B66" s="20"/>
-      <c r="C66" s="20"/>
-      <c r="D66" s="20"/>
-      <c r="E66" s="20"/>
-      <c r="F66" s="20"/>
-      <c r="G66" s="20"/>
-      <c r="H66" s="20"/>
-    </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A67" s="20"/>
-      <c r="B67" s="20"/>
-      <c r="C67" s="20"/>
-      <c r="D67" s="20"/>
-      <c r="E67" s="20"/>
-      <c r="F67" s="20"/>
-      <c r="G67" s="20"/>
-      <c r="H67" s="20"/>
-    </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A68" s="20"/>
-      <c r="B68" s="20"/>
-      <c r="C68" s="20"/>
-      <c r="D68" s="20"/>
-      <c r="E68" s="20"/>
-      <c r="F68" s="20"/>
-      <c r="G68" s="20"/>
-      <c r="H68" s="20"/>
-    </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A69" s="20"/>
-      <c r="B69" s="20"/>
-      <c r="C69" s="20"/>
-      <c r="D69" s="20"/>
-      <c r="E69" s="20"/>
-      <c r="F69" s="20"/>
-      <c r="G69" s="20"/>
+    <row r="69" spans="8:8" x14ac:dyDescent="0.2">
       <c r="H69" s="6"/>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A70" s="20"/>
-      <c r="B70" s="20"/>
-      <c r="C70" s="20"/>
-      <c r="D70" s="20"/>
-      <c r="E70" s="20"/>
-      <c r="F70" s="20"/>
-      <c r="G70" s="20"/>
+    <row r="70" spans="8:8" x14ac:dyDescent="0.2">
       <c r="H70" s="6"/>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A71" s="20"/>
-      <c r="B71" s="20"/>
-      <c r="C71" s="20"/>
-      <c r="D71" s="20"/>
-      <c r="E71" s="20"/>
-      <c r="F71" s="20"/>
-      <c r="G71" s="20"/>
+    <row r="71" spans="8:8" x14ac:dyDescent="0.2">
       <c r="H71" s="6"/>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A72" s="20"/>
-      <c r="B72" s="20"/>
-      <c r="C72" s="20"/>
-      <c r="D72" s="20"/>
-      <c r="E72" s="20"/>
-      <c r="F72" s="20"/>
-      <c r="G72" s="20"/>
+    <row r="72" spans="8:8" x14ac:dyDescent="0.2">
       <c r="H72" s="6"/>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A73" s="20"/>
-      <c r="B73" s="20"/>
-      <c r="C73" s="20"/>
-      <c r="D73" s="20"/>
-      <c r="E73" s="20"/>
-      <c r="F73" s="20"/>
-      <c r="G73" s="20"/>
+    <row r="73" spans="8:8" x14ac:dyDescent="0.2">
       <c r="H73" s="6"/>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A74" s="20"/>
-      <c r="B74" s="20"/>
-      <c r="C74" s="20"/>
-      <c r="D74" s="20"/>
-      <c r="E74" s="20"/>
-      <c r="F74" s="20"/>
-      <c r="G74" s="20"/>
+    <row r="74" spans="8:8" x14ac:dyDescent="0.2">
       <c r="H74" s="6"/>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A75" s="20"/>
-      <c r="B75" s="20"/>
-      <c r="C75" s="20"/>
-      <c r="D75" s="20"/>
-      <c r="E75" s="20"/>
-      <c r="F75" s="20"/>
-      <c r="G75" s="20"/>
+    <row r="75" spans="8:8" x14ac:dyDescent="0.2">
       <c r="H75" s="6"/>
-    </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A76" s="20"/>
-      <c r="B76" s="20"/>
-      <c r="C76" s="20"/>
-      <c r="D76" s="20"/>
-      <c r="E76" s="20"/>
-      <c r="F76" s="20"/>
-      <c r="G76" s="20"/>
-      <c r="H76" s="20"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2528,7 +2369,7 @@
         <v>29</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>136</v>
@@ -2584,7 +2425,7 @@
         <v>33</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C14" s="10" t="s">
         <v>136</v>
@@ -2598,7 +2439,7 @@
         <v>34</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C15" s="10" t="s">
         <v>136</v>
@@ -2640,7 +2481,7 @@
         <v>41</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C18" s="10" t="s">
         <v>136</v>

</xml_diff>